<commit_message>
everything from year 4
</commit_message>
<xml_diff>
--- a/ANUL4/sem2/th/lab2.xlsx
+++ b/ANUL4/sem2/th/lab2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\blabla\Downloads\uni\ANUL4\sem2\th\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11C0B1A9-3DD5-4CB9-9035-96D1A0FDE14E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{723A8721-E577-4FF9-9194-076CB1A4AE85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14415" yWindow="0" windowWidth="14385" windowHeight="15600" xr2:uid="{40BB519C-B9DD-4F0E-B812-73DE7F09E334}"/>
+    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{40BB519C-B9DD-4F0E-B812-73DE7F09E334}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="34">
   <si>
     <t>Nr.</t>
   </si>
@@ -119,6 +119,24 @@
   <si>
     <t>Calea</t>
   </si>
+  <si>
+    <t xml:space="preserve">D </t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>D'</t>
+  </si>
+  <si>
+    <t>7,8 - 9,10</t>
+  </si>
+  <si>
+    <t>6, 8 - 9,10</t>
+  </si>
+  <si>
+    <t>vid</t>
+  </si>
 </sst>
 </file>
 
@@ -147,7 +165,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -157,6 +175,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -188,12 +212,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -206,6 +227,15 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -522,33 +552,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFDAC4BD-4623-4CC8-9106-03ADDEBC9C2D}">
-  <dimension ref="A1:XFA18"/>
+  <dimension ref="A1:XFA37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="13" max="13" width="16.42578125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:16381" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2" t="s">
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="3" t="s">
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="6" t="s">
         <v>27</v>
       </c>
       <c r="N1" s="1"/>
@@ -16921,698 +16954,1272 @@
       <c r="XFA1" s="1"/>
     </row>
     <row r="2" spans="1:16381" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="3" t="s">
+      <c r="A2" s="6"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="3">
+      <c r="H2" s="2">
         <v>6</v>
       </c>
-      <c r="I2" s="3">
+      <c r="I2" s="2">
         <v>7</v>
       </c>
-      <c r="J2" s="3">
+      <c r="J2" s="2">
         <v>8</v>
       </c>
-      <c r="K2" s="3">
+      <c r="K2" s="2">
         <v>9</v>
       </c>
-      <c r="L2" s="3">
+      <c r="L2" s="2">
         <v>10</v>
       </c>
-      <c r="M2" s="2"/>
+      <c r="M2" s="6"/>
     </row>
     <row r="3" spans="1:16381" x14ac:dyDescent="0.25">
-      <c r="A3" s="4">
+      <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="4">
         <v>1</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="5">
         <v>0</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="4">
+      <c r="H3" s="3">
         <v>1</v>
       </c>
-      <c r="I3" s="4">
+      <c r="I3" s="3">
         <v>1</v>
       </c>
-      <c r="J3" s="4">
+      <c r="J3" s="3">
         <v>1</v>
       </c>
-      <c r="K3" s="4">
+      <c r="K3" s="3">
         <v>0</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3" s="3">
         <v>1</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="M3" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:16381" x14ac:dyDescent="0.25">
-      <c r="A4" s="4">
+      <c r="A4" s="3">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="4">
         <v>0</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="5">
         <v>0</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="3">
         <v>0</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="3">
         <v>1</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="3">
         <v>0</v>
       </c>
-      <c r="K4" s="4">
+      <c r="K4" s="3">
         <v>0</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="3">
         <v>0</v>
       </c>
-      <c r="M4" s="4" t="s">
+      <c r="M4" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:16381" x14ac:dyDescent="0.25">
-      <c r="A5" s="4">
+      <c r="A5" s="3">
         <v>3</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="4">
         <v>1</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="5">
         <v>1</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="5">
         <v>1</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="5">
         <v>1</v>
       </c>
-      <c r="H5" s="4">
+      <c r="H5" s="3">
         <v>1</v>
       </c>
-      <c r="I5" s="4">
+      <c r="I5" s="3">
         <v>0</v>
       </c>
-      <c r="J5" s="4">
+      <c r="J5" s="3">
         <v>0</v>
       </c>
-      <c r="K5" s="4">
+      <c r="K5" s="3">
         <v>0</v>
       </c>
-      <c r="L5" s="4">
+      <c r="L5" s="3">
         <v>0</v>
       </c>
-      <c r="M5" s="4" t="s">
+      <c r="M5" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:16381" x14ac:dyDescent="0.25">
-      <c r="A6" s="4">
+      <c r="A6" s="3">
         <v>4</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="4">
         <v>0</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="5">
         <v>1</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="5">
         <v>1</v>
       </c>
-      <c r="G6" s="6">
+      <c r="G6" s="5">
         <v>1</v>
       </c>
-      <c r="H6" s="4">
+      <c r="H6" s="3">
         <v>0</v>
       </c>
-      <c r="I6" s="4">
+      <c r="I6" s="3">
         <v>0</v>
       </c>
-      <c r="J6" s="4">
+      <c r="J6" s="3">
         <v>0</v>
       </c>
-      <c r="K6" s="4">
+      <c r="K6" s="3">
         <v>1</v>
       </c>
-      <c r="L6" s="4">
+      <c r="L6" s="3">
         <v>1</v>
       </c>
-      <c r="M6" s="4" t="s">
+      <c r="M6" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:16381" x14ac:dyDescent="0.25">
-      <c r="A7" s="4">
+      <c r="A7" s="3">
         <v>5</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="5">
         <v>1</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="4">
         <v>1</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="4">
+      <c r="H7" s="3">
         <v>0</v>
       </c>
-      <c r="I7" s="4">
+      <c r="I7" s="3">
         <v>1</v>
       </c>
-      <c r="J7" s="4">
+      <c r="J7" s="3">
         <v>0</v>
       </c>
-      <c r="K7" s="4">
+      <c r="K7" s="3">
         <v>0</v>
       </c>
-      <c r="L7" s="4">
+      <c r="L7" s="3">
         <v>0</v>
       </c>
-      <c r="M7" s="4" t="s">
+      <c r="M7" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:16381" x14ac:dyDescent="0.25">
-      <c r="A8" s="4">
+      <c r="A8" s="3">
         <v>6</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="5">
         <v>1</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="4">
         <v>0</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="4">
+      <c r="H8" s="3">
         <v>1</v>
       </c>
-      <c r="I8" s="4">
+      <c r="I8" s="3">
         <v>1</v>
       </c>
-      <c r="J8" s="4">
+      <c r="J8" s="3">
         <v>1</v>
       </c>
-      <c r="K8" s="4">
+      <c r="K8" s="3">
         <v>0</v>
       </c>
-      <c r="L8" s="4">
+      <c r="L8" s="3">
         <v>1</v>
       </c>
-      <c r="M8" s="4" t="s">
+      <c r="M8" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:16381" x14ac:dyDescent="0.25">
-      <c r="A9" s="4">
+      <c r="A9" s="3">
         <v>7</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="5">
         <v>1</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="5">
         <v>0</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="4">
         <v>1</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="5">
         <v>1</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="3">
         <v>1</v>
       </c>
-      <c r="I9" s="4">
+      <c r="I9" s="3">
         <v>0</v>
       </c>
-      <c r="J9" s="4">
+      <c r="J9" s="3">
         <v>0</v>
       </c>
-      <c r="K9" s="4">
+      <c r="K9" s="3">
         <v>0</v>
       </c>
-      <c r="L9" s="4">
+      <c r="L9" s="3">
         <v>0</v>
       </c>
-      <c r="M9" s="4" t="s">
+      <c r="M9" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:16381" x14ac:dyDescent="0.25">
-      <c r="A10" s="4">
+      <c r="A10" s="3">
         <v>8</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="5">
         <v>1</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="5">
         <v>0</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="4">
         <v>0</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="5">
         <v>1</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="G10" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H10" s="4">
+      <c r="H10" s="3">
         <v>1</v>
       </c>
-      <c r="I10" s="4">
+      <c r="I10" s="3">
         <v>1</v>
       </c>
-      <c r="J10" s="4">
+      <c r="J10" s="3">
         <v>1</v>
       </c>
-      <c r="K10" s="4">
+      <c r="K10" s="3">
         <v>0</v>
       </c>
-      <c r="L10" s="4">
+      <c r="L10" s="3">
         <v>1</v>
       </c>
-      <c r="M10" s="4" t="s">
+      <c r="M10" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:16381" x14ac:dyDescent="0.25">
-      <c r="A11" s="4">
+      <c r="A11" s="3">
         <v>9</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="5">
         <v>0</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="4">
         <v>1</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="5">
         <v>1</v>
       </c>
-      <c r="G11" s="6">
+      <c r="G11" s="5">
         <v>1</v>
       </c>
-      <c r="H11" s="4">
+      <c r="H11" s="3">
         <v>0</v>
       </c>
-      <c r="I11" s="4">
+      <c r="I11" s="3">
         <v>0</v>
       </c>
-      <c r="J11" s="4">
+      <c r="J11" s="3">
         <v>0</v>
       </c>
-      <c r="K11" s="4">
+      <c r="K11" s="3">
         <v>1</v>
       </c>
-      <c r="L11" s="4">
+      <c r="L11" s="3">
         <v>1</v>
       </c>
-      <c r="M11" s="4" t="s">
+      <c r="M11" s="3" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:16381" x14ac:dyDescent="0.25">
-      <c r="A12" s="4">
+      <c r="A12" s="3">
         <v>10</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="5">
         <v>0</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="4">
         <v>0</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="5">
         <v>1</v>
       </c>
-      <c r="G12" s="6">
+      <c r="G12" s="5">
         <v>1</v>
       </c>
-      <c r="H12" s="4">
+      <c r="H12" s="3">
         <v>0</v>
       </c>
-      <c r="I12" s="4">
+      <c r="I12" s="3">
         <v>1</v>
       </c>
-      <c r="J12" s="4">
+      <c r="J12" s="3">
         <v>0</v>
       </c>
-      <c r="K12" s="4">
+      <c r="K12" s="3">
         <v>0</v>
       </c>
-      <c r="L12" s="4">
+      <c r="L12" s="3">
         <v>0</v>
       </c>
-      <c r="M12" s="4" t="s">
+      <c r="M12" s="3" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:16381" x14ac:dyDescent="0.25">
-      <c r="A13" s="4">
+      <c r="A13" s="3">
         <v>11</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="5">
         <v>1</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="5">
         <v>0</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="5">
         <v>1</v>
       </c>
-      <c r="F13" s="5">
+      <c r="F13" s="4">
         <v>1</v>
       </c>
-      <c r="G13" s="6" t="s">
+      <c r="G13" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H13" s="4">
+      <c r="H13" s="3">
         <v>1</v>
       </c>
-      <c r="I13" s="4">
+      <c r="I13" s="3">
         <v>0</v>
       </c>
-      <c r="J13" s="4">
+      <c r="J13" s="3">
         <v>0</v>
       </c>
-      <c r="K13" s="4">
+      <c r="K13" s="3">
         <v>0</v>
       </c>
-      <c r="L13" s="4">
+      <c r="L13" s="3">
         <v>0</v>
       </c>
-      <c r="M13" s="4" t="s">
+      <c r="M13" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:16381" x14ac:dyDescent="0.25">
-      <c r="A14" s="4">
+      <c r="A14" s="3">
         <v>12</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="5">
         <v>1</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="5">
         <v>0</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="5">
         <v>1</v>
       </c>
-      <c r="F14" s="5">
+      <c r="F14" s="4">
         <v>0</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="G14" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H14" s="4">
+      <c r="H14" s="3">
         <v>1</v>
       </c>
-      <c r="I14" s="4">
+      <c r="I14" s="3">
         <v>1</v>
       </c>
-      <c r="J14" s="4">
+      <c r="J14" s="3">
         <v>1</v>
       </c>
-      <c r="K14" s="4">
+      <c r="K14" s="3">
         <v>0</v>
       </c>
-      <c r="L14" s="4">
+      <c r="L14" s="3">
         <v>1</v>
       </c>
-      <c r="M14" s="4" t="s">
+      <c r="M14" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:16381" x14ac:dyDescent="0.25">
-      <c r="A15" s="4">
+      <c r="A15" s="3">
         <v>13</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="6">
+      <c r="C15" s="5">
         <v>0</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="5">
         <v>1</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="4">
         <v>1</v>
       </c>
-      <c r="G15" s="6">
+      <c r="G15" s="5">
         <v>1</v>
       </c>
-      <c r="H15" s="4">
+      <c r="H15" s="3">
         <v>0</v>
       </c>
-      <c r="I15" s="4">
+      <c r="I15" s="3">
         <v>0</v>
       </c>
-      <c r="J15" s="4">
+      <c r="J15" s="3">
         <v>0</v>
       </c>
-      <c r="K15" s="4">
+      <c r="K15" s="3">
         <v>1</v>
       </c>
-      <c r="L15" s="4">
+      <c r="L15" s="3">
         <v>1</v>
       </c>
-      <c r="M15" s="4" t="s">
+      <c r="M15" s="3" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:16381" x14ac:dyDescent="0.25">
-      <c r="A16" s="4">
+      <c r="A16" s="3">
         <v>14</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="6">
+      <c r="C16" s="5">
         <v>0</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E16" s="6">
+      <c r="E16" s="5">
         <v>1</v>
       </c>
-      <c r="F16" s="5">
+      <c r="F16" s="4">
         <v>0</v>
       </c>
-      <c r="G16" s="6">
+      <c r="G16" s="5">
         <v>1</v>
       </c>
-      <c r="H16" s="4">
+      <c r="H16" s="3">
         <v>0</v>
       </c>
-      <c r="I16" s="4">
+      <c r="I16" s="3">
         <v>1</v>
       </c>
-      <c r="J16" s="4">
+      <c r="J16" s="3">
         <v>0</v>
       </c>
-      <c r="K16" s="4">
+      <c r="K16" s="3">
         <v>0</v>
       </c>
-      <c r="L16" s="4">
+      <c r="L16" s="3">
         <v>0</v>
       </c>
-      <c r="M16" s="4" t="s">
+      <c r="M16" s="3" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A17" s="4">
+      <c r="A17" s="3">
         <v>15</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C17" s="6">
+      <c r="C17" s="5">
         <v>0</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="5">
         <v>1</v>
       </c>
-      <c r="F17" s="6">
+      <c r="F17" s="5">
         <v>1</v>
       </c>
-      <c r="G17" s="5">
+      <c r="G17" s="4">
         <v>1</v>
       </c>
-      <c r="H17" s="4">
+      <c r="H17" s="3">
         <v>0</v>
       </c>
-      <c r="I17" s="4">
+      <c r="I17" s="3">
         <v>0</v>
       </c>
-      <c r="J17" s="4">
+      <c r="J17" s="3">
         <v>0</v>
       </c>
-      <c r="K17" s="4">
+      <c r="K17" s="3">
         <v>1</v>
       </c>
-      <c r="L17" s="4">
+      <c r="L17" s="3">
         <v>1</v>
       </c>
-      <c r="M17" s="4" t="s">
+      <c r="M17" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A18" s="4">
+      <c r="A18" s="3">
         <v>16</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C18" s="6">
+      <c r="C18" s="5">
         <v>0</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="5">
         <v>1</v>
       </c>
-      <c r="F18" s="6">
+      <c r="F18" s="5">
         <v>1</v>
       </c>
-      <c r="G18" s="5">
+      <c r="G18" s="4">
         <v>0</v>
       </c>
-      <c r="H18" s="4">
+      <c r="H18" s="3">
         <v>0</v>
       </c>
-      <c r="I18" s="4">
+      <c r="I18" s="3">
         <v>0</v>
       </c>
-      <c r="J18" s="4">
+      <c r="J18" s="3">
         <v>0</v>
       </c>
-      <c r="K18" s="4">
+      <c r="K18" s="3">
         <v>0</v>
       </c>
-      <c r="L18" s="4">
+      <c r="L18" s="3">
         <v>0</v>
       </c>
-      <c r="M18" s="4" t="s">
+      <c r="M18" s="3" t="s">
         <v>15</v>
       </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="I21" s="6"/>
+      <c r="J21" s="6"/>
+      <c r="K21" s="6"/>
+      <c r="L21" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="M21" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A22" s="6"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H22" s="2">
+        <v>6</v>
+      </c>
+      <c r="I22" s="2">
+        <v>7</v>
+      </c>
+      <c r="J22" s="2">
+        <v>8</v>
+      </c>
+      <c r="K22" s="2">
+        <v>9</v>
+      </c>
+      <c r="L22" s="2">
+        <v>10</v>
+      </c>
+      <c r="M22" s="6"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23" s="3">
+        <v>1</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D23" s="5">
+        <v>0</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I23" s="5">
+        <v>1</v>
+      </c>
+      <c r="J23" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="K23" s="5">
+        <v>0</v>
+      </c>
+      <c r="L23" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="M23" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A24" s="3">
+        <v>2</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" s="5">
+        <v>1</v>
+      </c>
+      <c r="F24" s="5">
+        <v>1</v>
+      </c>
+      <c r="G24" s="5">
+        <v>1</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I24" s="5">
+        <v>0</v>
+      </c>
+      <c r="J24" s="5">
+        <v>0</v>
+      </c>
+      <c r="K24" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="L24" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="M24" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A25" s="3">
+        <v>3</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D25" s="5">
+        <v>0</v>
+      </c>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5">
+        <v>1</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J25" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="K25" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="L25" s="5">
+        <v>1</v>
+      </c>
+      <c r="M25" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A26" s="3">
+        <v>4</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C26" s="7">
+        <v>1</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" s="5">
+        <v>0</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I26" s="5">
+        <v>1</v>
+      </c>
+      <c r="J26" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="K26" s="5">
+        <v>0</v>
+      </c>
+      <c r="L26" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="M26" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A27" s="3">
+        <v>5</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" s="5">
+        <v>1</v>
+      </c>
+      <c r="D27" s="7">
+        <v>0</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F27" s="5">
+        <v>1</v>
+      </c>
+      <c r="G27" s="5">
+        <v>0</v>
+      </c>
+      <c r="H27" s="5">
+        <v>1</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J27" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="K27" s="5">
+        <v>0</v>
+      </c>
+      <c r="L27" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="M27" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A28" s="3">
+        <v>6</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" s="5">
+        <v>0</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F28" s="5">
+        <v>1</v>
+      </c>
+      <c r="G28" s="5">
+        <v>1</v>
+      </c>
+      <c r="H28" s="5">
+        <v>0</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J28" s="5">
+        <v>0</v>
+      </c>
+      <c r="K28" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="L28" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="M28" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A29" s="3">
+        <v>7</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D29" s="5">
+        <v>0</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F29" s="5">
+        <v>1</v>
+      </c>
+      <c r="G29" s="5">
+        <v>1</v>
+      </c>
+      <c r="H29" s="5">
+        <v>1</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J29" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="K29" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L29" s="5">
+        <v>1</v>
+      </c>
+      <c r="M29" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A30" s="3">
+        <v>8</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C30" s="5">
+        <v>1</v>
+      </c>
+      <c r="D30" s="5">
+        <v>0</v>
+      </c>
+      <c r="E30" s="7">
+        <v>1</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H30" s="5">
+        <v>1</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J30" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="K30" s="5">
+        <v>0</v>
+      </c>
+      <c r="L30" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="M30" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A31" s="3">
+        <v>9</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C31" s="5">
+        <v>0</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E31" s="7">
+        <v>1</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="G31" s="5">
+        <v>1</v>
+      </c>
+      <c r="H31" s="5">
+        <v>0</v>
+      </c>
+      <c r="I31" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J31" s="5">
+        <v>0</v>
+      </c>
+      <c r="K31" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L31" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="M31" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A32" s="3">
+        <v>10</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D32" s="5">
+        <v>0</v>
+      </c>
+      <c r="E32" s="5">
+        <v>1</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="G32" s="5">
+        <v>1</v>
+      </c>
+      <c r="H32" s="5">
+        <v>1</v>
+      </c>
+      <c r="I32" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J32" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="K32" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L32" s="5">
+        <v>1</v>
+      </c>
+      <c r="M32" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A33" s="3">
+        <v>11</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C33" s="5">
+        <v>0</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E33" s="5">
+        <v>1</v>
+      </c>
+      <c r="F33" s="7">
+        <v>1</v>
+      </c>
+      <c r="G33" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="H33" s="5">
+        <v>0</v>
+      </c>
+      <c r="I33" s="5">
+        <v>0</v>
+      </c>
+      <c r="J33" s="5">
+        <v>0</v>
+      </c>
+      <c r="K33" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L33" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="M33" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A34" s="3"/>
+      <c r="B34" s="3"/>
+      <c r="C34" s="5"/>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="7"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="5"/>
+      <c r="I34" s="5"/>
+      <c r="J34" s="5"/>
+      <c r="K34" s="5"/>
+      <c r="L34" s="5"/>
+      <c r="M34" s="3"/>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A35" s="3"/>
+      <c r="B35" s="3"/>
+      <c r="C35" s="5"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="7"/>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5"/>
+      <c r="I35" s="5"/>
+      <c r="J35" s="5"/>
+      <c r="K35" s="5"/>
+      <c r="L35" s="5"/>
+      <c r="M35" s="3"/>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A36" s="3"/>
+      <c r="B36" s="3"/>
+      <c r="C36" s="5"/>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="7"/>
+      <c r="H36" s="5"/>
+      <c r="I36" s="5"/>
+      <c r="J36" s="5"/>
+      <c r="K36" s="5"/>
+      <c r="L36" s="5"/>
+      <c r="M36" s="3"/>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A37" s="3"/>
+      <c r="B37" s="3"/>
+      <c r="C37" s="5"/>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="7"/>
+      <c r="H37" s="5"/>
+      <c r="I37" s="5"/>
+      <c r="J37" s="5"/>
+      <c r="K37" s="5"/>
+      <c r="L37" s="5"/>
+      <c r="M37" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="10">
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:G21"/>
+    <mergeCell ref="H21:K21"/>
+    <mergeCell ref="M21:M22"/>
     <mergeCell ref="H1:K1"/>
     <mergeCell ref="C1:G1"/>
     <mergeCell ref="M1:M2"/>

</xml_diff>